<commit_message>
Edited some management data based on paper reviews
</commit_message>
<xml_diff>
--- a/Data/2002_F105_CO_FISE/2002_F105_CO_FISE_Management.xlsx
+++ b/Data/2002_F105_CO_FISE/2002_F105_CO_FISE_Management.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\mnt\Data1\USDA-ALARC\GIS\PDI project\cottondata\Data\2002_F105_CO_FISE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE5F03A-C162-45DE-B4F1-FD3BFBC12491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11DE351-3FF1-4C88-B844-C45C3E1D4F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1545" yWindow="-23595" windowWidth="17865" windowHeight="22530" activeTab="3" xr2:uid="{13866AC3-1731-43DF-8B05-09EFA100F22B}"/>
+    <workbookView xWindow="-975" yWindow="-28020" windowWidth="17310" windowHeight="16335" activeTab="3" xr2:uid="{13866AC3-1731-43DF-8B05-09EFA100F22B}"/>
   </bookViews>
   <sheets>
     <sheet name="Irrigation" sheetId="2" r:id="rId1"/>
@@ -42894,7 +42894,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80D165EC-9026-46FC-B0FA-7D576B091D93}">
-  <dimension ref="A1:AP6"/>
+  <dimension ref="A1:AP7"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:42" x14ac:dyDescent="0.2">
@@ -43030,55 +43030,127 @@
         <v>2002</v>
       </c>
       <c r="B2">
-        <v>155</v>
+        <v>100</v>
       </c>
       <c r="C2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="D2">
+        <v>36</v>
       </c>
       <c r="E2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="F2">
+        <v>36</v>
+      </c>
+      <c r="G2">
+        <v>36</v>
       </c>
       <c r="H2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="I2">
+        <v>36</v>
       </c>
       <c r="J2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="K2">
+        <v>36</v>
       </c>
       <c r="L2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="M2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="N2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="O2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="P2">
+        <v>36</v>
+      </c>
+      <c r="Q2">
+        <v>36</v>
+      </c>
+      <c r="R2">
+        <v>36</v>
+      </c>
+      <c r="S2">
+        <v>36</v>
+      </c>
+      <c r="T2">
+        <v>36</v>
+      </c>
+      <c r="U2">
+        <v>36</v>
+      </c>
+      <c r="V2">
+        <v>36</v>
       </c>
       <c r="W2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="X2">
+        <v>36</v>
       </c>
       <c r="Y2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="Z2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="AA2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="AB2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="AC2">
+        <v>36</v>
       </c>
       <c r="AD2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="AE2">
+        <v>36</v>
       </c>
       <c r="AF2">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="AG2">
-        <v>84</v>
+        <v>36</v>
+      </c>
+      <c r="AH2">
+        <v>36</v>
+      </c>
+      <c r="AI2">
+        <v>36</v>
+      </c>
+      <c r="AJ2">
+        <v>36</v>
+      </c>
+      <c r="AK2">
+        <v>36</v>
+      </c>
+      <c r="AL2">
+        <v>36</v>
+      </c>
+      <c r="AM2">
+        <v>36</v>
+      </c>
+      <c r="AN2">
+        <v>36</v>
+      </c>
+      <c r="AO2">
+        <v>36</v>
+      </c>
+      <c r="AP2">
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:42" x14ac:dyDescent="0.2">
@@ -43086,13 +43158,55 @@
         <v>2002</v>
       </c>
       <c r="B3">
-        <v>188</v>
+        <v>155</v>
+      </c>
+      <c r="C3">
+        <v>84</v>
+      </c>
+      <c r="E3">
+        <v>84</v>
+      </c>
+      <c r="H3">
+        <v>84</v>
+      </c>
+      <c r="J3">
+        <v>84</v>
+      </c>
+      <c r="L3">
+        <v>84</v>
+      </c>
+      <c r="M3">
+        <v>84</v>
       </c>
       <c r="N3">
-        <v>56</v>
+        <v>84</v>
+      </c>
+      <c r="O3">
+        <v>84</v>
       </c>
       <c r="W3">
-        <v>56</v>
+        <v>84</v>
+      </c>
+      <c r="Y3">
+        <v>84</v>
+      </c>
+      <c r="Z3">
+        <v>84</v>
+      </c>
+      <c r="AA3">
+        <v>84</v>
+      </c>
+      <c r="AB3">
+        <v>84</v>
+      </c>
+      <c r="AD3">
+        <v>84</v>
+      </c>
+      <c r="AF3">
+        <v>84</v>
+      </c>
+      <c r="AG3">
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:42" x14ac:dyDescent="0.2">
@@ -43100,30 +43214,12 @@
         <v>2002</v>
       </c>
       <c r="B4">
-        <v>189</v>
-      </c>
-      <c r="C4">
+        <v>188</v>
+      </c>
+      <c r="N4">
         <v>56</v>
       </c>
-      <c r="E4">
-        <v>56</v>
-      </c>
-      <c r="J4">
-        <v>56</v>
-      </c>
-      <c r="M4">
-        <v>56</v>
-      </c>
-      <c r="O4">
-        <v>56</v>
-      </c>
-      <c r="Z4">
-        <v>56</v>
-      </c>
-      <c r="AD4">
-        <v>56</v>
-      </c>
-      <c r="AF4">
+      <c r="W4">
         <v>56</v>
       </c>
     </row>
@@ -43132,18 +43228,30 @@
         <v>2002</v>
       </c>
       <c r="B5">
-        <v>193</v>
-      </c>
-      <c r="H5">
+        <v>189</v>
+      </c>
+      <c r="C5">
         <v>56</v>
       </c>
-      <c r="L5">
+      <c r="E5">
         <v>56</v>
       </c>
-      <c r="Y5">
+      <c r="J5">
         <v>56</v>
       </c>
-      <c r="AB5">
+      <c r="M5">
+        <v>56</v>
+      </c>
+      <c r="O5">
+        <v>56</v>
+      </c>
+      <c r="Z5">
+        <v>56</v>
+      </c>
+      <c r="AD5">
+        <v>56</v>
+      </c>
+      <c r="AF5">
         <v>56</v>
       </c>
     </row>
@@ -43152,12 +43260,32 @@
         <v>2002</v>
       </c>
       <c r="B6">
+        <v>193</v>
+      </c>
+      <c r="H6">
+        <v>56</v>
+      </c>
+      <c r="L6">
+        <v>56</v>
+      </c>
+      <c r="Y6">
+        <v>56</v>
+      </c>
+      <c r="AB6">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>2002</v>
+      </c>
+      <c r="B7">
         <v>195</v>
       </c>
-      <c r="AA6">
+      <c r="AA7">
         <v>56</v>
       </c>
-      <c r="AG6">
+      <c r="AG7">
         <v>56</v>
       </c>
     </row>

</xml_diff>